<commit_message>
changes mainly in package.json
</commit_message>
<xml_diff>
--- a/Journey/Moms Adopting Moms.xlsx
+++ b/Journey/Moms Adopting Moms.xlsx
@@ -19,7 +19,7 @@
     <sheet name="Supporters" sheetId="4" r:id="rId4"/>
     <sheet name="Case Workers" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t>Parent ID</t>
   </si>
@@ -150,12 +150,18 @@
     <t>Venuswoman</t>
   </si>
   <si>
+    <t>StepE-3</t>
+  </si>
+  <si>
     <t>Mary</t>
   </si>
   <si>
     <t>Peachtree</t>
   </si>
   <si>
+    <t>FirstStep</t>
+  </si>
+  <si>
     <t>Case Worker 1</t>
   </si>
   <si>
@@ -193,16 +199,14 @@
   </si>
   <si>
     <t>Cell Phone</t>
-  </si>
-  <si>
-    <t>FirstStep</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -553,42 +557,42 @@
   <dimension ref="A1:AH3"/>
   <sheetFormatPr defaultColWidth="15.265625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.73046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.53125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.1328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.53125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.3984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.53125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.73046875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.53125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.1328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.53125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.265625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.1328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="17.86328125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7.86328125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="17.73046875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.86328125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.53125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.73046875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="15.1328125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="9.3984375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="8.3984375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="9" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="18.53125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="10.265625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="25.86328125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="14.3984375" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="14.73046875" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="18.86328125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="22.265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="1" width="9.1328125" customWidth="1"/>
+    <col min="2" max="2" bestFit="1" width="19.73046875" customWidth="1"/>
+    <col min="3" max="3" bestFit="1" width="12.1328125" customWidth="1"/>
+    <col min="4" max="4" bestFit="1" width="10.53125" customWidth="1"/>
+    <col min="5" max="5" bestFit="1" width="10.1328125" customWidth="1"/>
+    <col min="6" max="6" bestFit="1" width="14.53125" customWidth="1"/>
+    <col min="7" max="7" bestFit="1" width="4.3984375" customWidth="1"/>
+    <col min="8" max="8" bestFit="1" width="5.53125" customWidth="1"/>
+    <col min="9" max="9" bestFit="1" width="8.73046875" customWidth="1"/>
+    <col min="10" max="10" bestFit="1" width="18.53125" customWidth="1"/>
+    <col min="11" max="11" bestFit="1" width="12.1328125" customWidth="1"/>
+    <col min="12" max="12" bestFit="1" width="13.53125" customWidth="1"/>
+    <col min="13" max="13" bestFit="1" width="12.265625" customWidth="1"/>
+    <col min="14" max="14" bestFit="1" width="10.3984375" customWidth="1"/>
+    <col min="15" max="15" bestFit="1" width="16.1328125" customWidth="1"/>
+    <col min="16" max="16" bestFit="1" width="17.86328125" customWidth="1"/>
+    <col min="17" max="17" bestFit="1" width="7.86328125" customWidth="1"/>
+    <col min="18" max="18" bestFit="1" width="17.73046875" customWidth="1"/>
+    <col min="19" max="19" bestFit="1" width="11.86328125" customWidth="1"/>
+    <col min="20" max="20" bestFit="1" width="12.53125" customWidth="1"/>
+    <col min="21" max="21" bestFit="1" width="13.86328125" customWidth="1"/>
+    <col min="22" max="22" bestFit="1" width="6.73046875" customWidth="1"/>
+    <col min="23" max="23" bestFit="1" width="15.1328125" customWidth="1"/>
+    <col min="24" max="24" bestFit="1" width="9.3984375" customWidth="1"/>
+    <col min="25" max="25" bestFit="1" width="8.3984375" customWidth="1"/>
+    <col min="26" max="26" bestFit="1" width="9" customWidth="1"/>
+    <col min="27" max="27" bestFit="1" width="18.53125" customWidth="1"/>
+    <col min="28" max="28" bestFit="1" width="10.265625" customWidth="1"/>
+    <col min="29" max="29" bestFit="1" width="25.86328125" customWidth="1"/>
+    <col min="30" max="30" bestFit="1" width="14.3984375" customWidth="1"/>
+    <col min="31" max="31" bestFit="1" width="14.73046875" customWidth="1"/>
+    <col min="32" max="32" bestFit="1" width="18.86328125" customWidth="1"/>
+    <col min="33" max="33" bestFit="1" width="22.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -692,43 +696,44 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A2">
+    <row r="2">
+      <c r="A2" s="0">
         <v>12345</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="0" t="s">
         <v>34</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="0">
         <v>48201</v>
       </c>
-      <c r="AH2" t="s">
-        <v>51</v>
+      <c r="AH2" s="0" t="s">
+        <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A3">
+    <row r="3">
+      <c r="A3" s="0">
         <v>67890</v>
       </c>
-      <c r="D3" t="s">
-        <v>36</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="D3" s="0" t="s">
         <v>37</v>
       </c>
-      <c r="I3">
+      <c r="E3" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" s="0">
         <v>30303</v>
       </c>
-      <c r="AH3" t="s">
-        <v>51</v>
+      <c r="AH3" s="0" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
@@ -738,48 +743,48 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="5" width="14.53125" customWidth="1"/>
-    <col min="6" max="6" width="10.53125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.1328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.53125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.3984375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.53125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.73046875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.53125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.1328125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.53125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="30" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="32.3984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.1328125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="17.86328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="7.86328125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.73046875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.86328125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.53125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="6.73046875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="15.1328125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="25.86328125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="14.3984375" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="14.73046875" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="18.86328125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="22.265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" bestFit="1" width="10.53125" customWidth="1"/>
+    <col min="7" max="7" bestFit="1" width="10.1328125" customWidth="1"/>
+    <col min="8" max="8" bestFit="1" width="14.53125" customWidth="1"/>
+    <col min="9" max="9" bestFit="1" width="4.3984375" customWidth="1"/>
+    <col min="10" max="10" bestFit="1" width="5.53125" customWidth="1"/>
+    <col min="11" max="11" bestFit="1" width="8.73046875" customWidth="1"/>
+    <col min="12" max="12" bestFit="1" width="18.53125" customWidth="1"/>
+    <col min="13" max="13" bestFit="1" width="12.1328125" customWidth="1"/>
+    <col min="14" max="14" bestFit="1" width="13.53125" customWidth="1"/>
+    <col min="15" max="15" bestFit="1" width="30" customWidth="1"/>
+    <col min="16" max="16" bestFit="1" width="32.3984375" customWidth="1"/>
+    <col min="17" max="17" bestFit="1" width="16.1328125" customWidth="1"/>
+    <col min="18" max="18" bestFit="1" width="17.86328125" customWidth="1"/>
+    <col min="19" max="19" bestFit="1" width="7.86328125" customWidth="1"/>
+    <col min="20" max="20" bestFit="1" width="17.73046875" customWidth="1"/>
+    <col min="21" max="21" bestFit="1" width="11.86328125" customWidth="1"/>
+    <col min="22" max="22" bestFit="1" width="12.53125" customWidth="1"/>
+    <col min="23" max="23" bestFit="1" width="13.86328125" customWidth="1"/>
+    <col min="24" max="24" bestFit="1" width="6.73046875" customWidth="1"/>
+    <col min="25" max="25" bestFit="1" width="15.1328125" customWidth="1"/>
+    <col min="26" max="26" bestFit="1" width="25.86328125" customWidth="1"/>
+    <col min="27" max="27" bestFit="1" width="14.3984375" customWidth="1"/>
+    <col min="28" max="28" bestFit="1" width="14.73046875" customWidth="1"/>
+    <col min="29" max="29" bestFit="1" width="18.86328125" customWidth="1"/>
+    <col min="30" max="30" bestFit="1" width="22.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -809,56 +814,57 @@
         <v>11</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
@@ -867,22 +873,22 @@
   <dimension ref="A1:AD1"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="10.53125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.1328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.53125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.3984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.53125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.73046875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.53125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.1328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.53125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.3984375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.1328125" bestFit="1" customWidth="1"/>
-    <col min="17" max="30" width="1.3984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="1" width="10.53125" customWidth="1"/>
+    <col min="2" max="2" bestFit="1" width="10.1328125" customWidth="1"/>
+    <col min="3" max="3" bestFit="1" width="14.53125" customWidth="1"/>
+    <col min="4" max="4" bestFit="1" width="4.3984375" customWidth="1"/>
+    <col min="5" max="5" bestFit="1" width="5.53125" customWidth="1"/>
+    <col min="6" max="6" bestFit="1" width="8.73046875" customWidth="1"/>
+    <col min="7" max="7" bestFit="1" width="18.53125" customWidth="1"/>
+    <col min="8" max="8" bestFit="1" width="12.1328125" customWidth="1"/>
+    <col min="9" max="9" bestFit="1" width="13.53125" customWidth="1"/>
+    <col min="10" max="10" bestFit="1" width="14" customWidth="1"/>
+    <col min="11" max="11" bestFit="1" width="13.3984375" customWidth="1"/>
+    <col min="12" max="12" bestFit="1" width="12.1328125" customWidth="1"/>
+    <col min="17" max="30" bestFit="1" width="1.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -911,59 +917,60 @@
         <v>11</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
@@ -972,22 +979,22 @@
   <dimension ref="A1:AD1"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="10.53125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.1328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.53125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.3984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.53125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.73046875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.53125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.1328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.53125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.3984375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.1328125" bestFit="1" customWidth="1"/>
-    <col min="17" max="30" width="1.3984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="1" width="10.53125" customWidth="1"/>
+    <col min="2" max="2" bestFit="1" width="10.1328125" customWidth="1"/>
+    <col min="3" max="3" bestFit="1" width="14.53125" customWidth="1"/>
+    <col min="4" max="4" bestFit="1" width="4.3984375" customWidth="1"/>
+    <col min="5" max="5" bestFit="1" width="5.53125" customWidth="1"/>
+    <col min="6" max="6" bestFit="1" width="8.73046875" customWidth="1"/>
+    <col min="7" max="7" bestFit="1" width="18.53125" customWidth="1"/>
+    <col min="8" max="8" bestFit="1" width="12.1328125" customWidth="1"/>
+    <col min="9" max="9" bestFit="1" width="13.53125" customWidth="1"/>
+    <col min="10" max="10" bestFit="1" width="14" customWidth="1"/>
+    <col min="11" max="11" bestFit="1" width="13.3984375" customWidth="1"/>
+    <col min="12" max="12" bestFit="1" width="12.1328125" customWidth="1"/>
+    <col min="17" max="30" bestFit="1" width="1.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1016,53 +1023,54 @@
         <v>11</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
@@ -1071,36 +1079,37 @@
   <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.53125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.1328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.86328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.53125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.53125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="1" width="7.265625" customWidth="1"/>
+    <col min="2" max="2" bestFit="1" width="10.53125" customWidth="1"/>
+    <col min="3" max="3" bestFit="1" width="10.1328125" customWidth="1"/>
+    <col min="4" max="4" bestFit="1" width="11.86328125" customWidth="1"/>
+    <col min="5" max="5" bestFit="1" width="10.53125" customWidth="1"/>
+    <col min="6" max="6" bestFit="1" width="13.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="D1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="D1" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" s="0" t="s">
         <v>11</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 

</xml_diff>